<commit_message>
XLSX: Additional infos in Worksheet "README"
</commit_message>
<xml_diff>
--- a/input-files/new-category-names/DLE-2024-new-category-names.xlsx
+++ b/input-files/new-category-names/DLE-2024-new-category-names.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DATA\SW_DATA\Python-Proj\database-toolkit\input-files\new-category-names\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C853C292-A80F-42C7-A5B0-6CE919FB9C7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D98FD0F0-B9A2-4BC8-91EA-76CA684666F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="1056" windowWidth="11256" windowHeight="11184" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="178">
   <si>
     <t>NA1</t>
   </si>
@@ -549,13 +549,19 @@
   </si>
   <si>
     <t>NA2</t>
+  </si>
+  <si>
+    <t>Achtung</t>
+  </si>
+  <si>
+    <t>Name des Reiters "Kategorie-Namen" darf nicht geändert werden</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -597,6 +603,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -618,13 +632,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -929,7 +944,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.77734375" customWidth="1"/>
@@ -1007,6 +1022,16 @@
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>170</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="6" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Excels mit neuen Kategorie-Namen für DL-2024
</commit_message>
<xml_diff>
--- a/input-files/new-category-names/DLE-2024-new-category-names.xlsx
+++ b/input-files/new-category-names/DLE-2024-new-category-names.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DATA\SW_DATA\Python-Proj\database-toolkit\input-files\new-category-names\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D98FD0F0-B9A2-4BC8-91EA-76CA684666F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B054A44-DE1D-43A8-9846-6EBC735ABD42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="184">
   <si>
     <t>NA1</t>
   </si>
@@ -278,138 +278,6 @@
     <t>Code</t>
   </si>
   <si>
-    <t>01.1. Mathematische Grundkenntnisse (3.1.1)</t>
-  </si>
-  <si>
-    <t>01.2. Grössen und Einheiten (3.1.2 + 4.1.2)</t>
-  </si>
-  <si>
-    <t>01.3. Binäres Zahlensystem (4.1.2)</t>
-  </si>
-  <si>
-    <t>02.1. Leiter, Halbleiter und Isolator (3.2.1)</t>
-  </si>
-  <si>
-    <t>02.2. Strom- und Spannungsquellen (3.2.2)</t>
-  </si>
-  <si>
-    <t>02.3. Elektromagnetisches Feld (3.2.3 + 4.2.1/2/3)</t>
-  </si>
-  <si>
-    <t>02.4. Sinusförmige Signale (3.2.4 + 4.2.4)</t>
-  </si>
-  <si>
-    <t>02.5. Ohmsches Gesetz und  Stromkreis (3.2.5 + 3.2.7)</t>
-  </si>
-  <si>
-    <t>02.6. Leistung (3.2.6 + 4.2.5)</t>
-  </si>
-  <si>
-    <t>03.1. Widerstand (3.3.1 + 4.3.1)</t>
-  </si>
-  <si>
-    <t>03.2. Kondensator (3.3.2 + 4.3.2)</t>
-  </si>
-  <si>
-    <t>03.3. Spule (3.3.3 + 4.3.3)</t>
-  </si>
-  <si>
-    <t>03.4. Diode (3.3.4 + 4.3.5)</t>
-  </si>
-  <si>
-    <t>04.1. Reihen- und Parallelschaltung (4.4.1)</t>
-  </si>
-  <si>
-    <t>04.2. Schwingkreise und Filter (4.4.2)</t>
-  </si>
-  <si>
-    <t>04.3. Strom- und Spannungsversorgung (3.4.1 + 4.4.3)</t>
-  </si>
-  <si>
-    <t>04.4. Verstärker (4.4.4)</t>
-  </si>
-  <si>
-    <t>04.5. Oszillator (3.4.2 + 4.4.5)</t>
-  </si>
-  <si>
-    <t>05.1. Modulation allgemein (3.5.1 + 4.5.1)</t>
-  </si>
-  <si>
-    <t>05.2. Amplitudenmodulation AM, SSB, CW (3.5.2 + 4.5.2)</t>
-  </si>
-  <si>
-    <t>05.3. Frequenz- und Phasenmodulation (3.5.3 + 4.5.3)</t>
-  </si>
-  <si>
-    <t>05.4. Digitale Übertragungsverfahren (3.5.4 + 4.5.4)</t>
-  </si>
-  <si>
-    <t>06.3. Empfängerstufen (3.6.3 + 4.6.2)</t>
-  </si>
-  <si>
-    <t>06.1. Transceiver (3.6.1)</t>
-  </si>
-  <si>
-    <t>06.2. Empfänger (3.6.2 + 4.6.1)</t>
-  </si>
-  <si>
-    <t>06.4. Sender und Senderstufen (3.6.4 + 4.6.3)</t>
-  </si>
-  <si>
-    <t>06.5. Leistungsverstärker (4.6.4)</t>
-  </si>
-  <si>
-    <t>06.6. Konverter und Transverter (4.6.5)</t>
-  </si>
-  <si>
-    <t>06.7. Digitale Signalverarbeitung (4.6.6)</t>
-  </si>
-  <si>
-    <t>07.1. Antennen (3.7.1 + 4.7.1)</t>
-  </si>
-  <si>
-    <t>07.2. Antennenmerkmale (4.7.2)</t>
-  </si>
-  <si>
-    <t>07.3. Übertragungsleitungen (3.7.2 + 4.7.3)</t>
-  </si>
-  <si>
-    <t>07.5. Strahlungsleistung  (3.7.4 + 4.7.5)</t>
-  </si>
-  <si>
-    <t>07.4. Anpassung usw. (3.7.3)</t>
-  </si>
-  <si>
-    <t>08.1. Ionosphäre (3.8.1 + 4.8.1)</t>
-  </si>
-  <si>
-    <t>08.2. Kurzwellenausbreitung (3.8.2 + 4.8.2)</t>
-  </si>
-  <si>
-    <t>08.3. Wellenausbreitung oberhalb 30 MHz (3.8.3 + 4.8.3)</t>
-  </si>
-  <si>
-    <t>09.1. Strom- und Spannungsmessgeräte (3.9.1 + 4.9.1)</t>
-  </si>
-  <si>
-    <t>09.2. Stehwellenmessgerät (3.9.2 + 4.9.4)</t>
-  </si>
-  <si>
-    <t>09.3. Vektorieller Netzwerk Analysator (4.9.2)</t>
-  </si>
-  <si>
-    <t>09.4. Frequenzmessung (3.9.3 + 4.9.5)</t>
-  </si>
-  <si>
-    <t>09.5. Oszilloskop (3.9.4 + 4.9.3)</t>
-  </si>
-  <si>
-    <t>10.1. Störungen elektronischer Geräte (3.10.1 + 4.10.1)</t>
-  </si>
-  <si>
-    <t>10.2. Unerwünschte Aussendungen (3.10.2 + 4.10.2)</t>
-  </si>
-  <si>
     <t>01. Math. Grundkenntnisse und Grössen</t>
   </si>
   <si>
@@ -428,9 +296,6 @@
     <t>06. Sender und Empfänger</t>
   </si>
   <si>
-    <t>07. Antennen und Übertragungsleitunggen</t>
-  </si>
-  <si>
     <t>08. Wellenausbreitung und Ionosphäre</t>
   </si>
   <si>
@@ -443,15 +308,6 @@
     <t>11. Sicherheit</t>
   </si>
   <si>
-    <t>10.3. Störfestigkeit (3.11.1)</t>
-  </si>
-  <si>
-    <t>11.1. Schutz von Personen (3.11.2 + 4.11.1)</t>
-  </si>
-  <si>
-    <t>11.2. Sicherheit (3.11.3 + 4.11.2)</t>
-  </si>
-  <si>
     <t>10. Messungen und Messinstrumente</t>
   </si>
   <si>
@@ -497,12 +353,6 @@
     <t>14. Sicherheit</t>
   </si>
   <si>
-    <t>03.5. Übertrager und Transformatoren (4.3.4)</t>
-  </si>
-  <si>
-    <t>03.6. Transistor (3.3.5 + 4.3.6)</t>
-  </si>
-  <si>
     <t>Hauptkategorie</t>
   </si>
   <si>
@@ -515,33 +365,15 @@
     <t>= Erste drei Buchstaben der 'Question-ID'. Diese ist eindeutig pro Unterkapitel _UND_ Klasse.</t>
   </si>
   <si>
-    <t>Hauptkapitel</t>
-  </si>
-  <si>
     <t>= orientiert sich nach den Kapiteln im off. Fragenkatalog  DL-2024 der BNetzA.</t>
   </si>
   <si>
-    <t>Unterkapitel</t>
-  </si>
-  <si>
     <t>= orientiert sich nach den Unterkapiteln im off. Fragenkatalog DL-2024 der BNetzA.</t>
   </si>
   <si>
     <t>Spalten</t>
   </si>
   <si>
-    <t>Aufbau</t>
-  </si>
-  <si>
-    <t>mehrheitlich mit identischen Namen. Daher ist eine gemeinsame Gliederung aller N- und E-Fragen möglich.</t>
-  </si>
-  <si>
-    <t>Die Einteilung in Kapitel und Unterkapitel ist bei den Technik-Prüfungsfragen nach dem gleichen Konzept und</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prüfungsteil "Technik" der Klasse N und E (Entry-License und Novice-License) </t>
-  </si>
-  <si>
     <t>aus dem Prüfungsfragenkatalog DL-2024 der BNetzA Deutschland.</t>
   </si>
   <si>
@@ -554,14 +386,200 @@
     <t>Achtung</t>
   </si>
   <si>
-    <t>Name des Reiters "Kategorie-Namen" darf nicht geändert werden</t>
+    <t>01.1a. Mathematische Grundkenntnisse (3.1.1)</t>
+  </si>
+  <si>
+    <t>01.2a. Grössen und Einheiten (3.1.2 + 4.1.2)</t>
+  </si>
+  <si>
+    <t>01.3a. Binäres Zahlensystem (4.1.2)</t>
+  </si>
+  <si>
+    <t>02.1a. Leiter, Halbleiter und Isolator (3.2.1)</t>
+  </si>
+  <si>
+    <t>02.2a. Strom- und Spannungsquellen (3.2.2)</t>
+  </si>
+  <si>
+    <t>02.3a. Elektromagnetisches Feld (3.2.3 + 4.2.1/2/3)</t>
+  </si>
+  <si>
+    <t>02.4a. Sinusförmige Signale (3.2.4 + 4.2.4)</t>
+  </si>
+  <si>
+    <t>03.1a. Widerstand (3.3.1 + 4.3.1)</t>
+  </si>
+  <si>
+    <t>03.2a. Kondensator (3.3.2 + 4.3.2)</t>
+  </si>
+  <si>
+    <t>03.3a. Spule (3.3.3 + 4.3.3)</t>
+  </si>
+  <si>
+    <t>03.6a. Transistor (3.3.5 + 4.3.6)</t>
+  </si>
+  <si>
+    <t>04.1a. Reihen- und Parallelschaltung (4.4.1)</t>
+  </si>
+  <si>
+    <t>04.2a. Schwingkreise und Filter (4.4.2)</t>
+  </si>
+  <si>
+    <t>04.3a. Strom- und Spannungsversorgung (3.4.1 + 4.4.3)</t>
+  </si>
+  <si>
+    <t>04.4a. Verstärker (4.4.4)</t>
+  </si>
+  <si>
+    <t>05.1a. Modulation allgemein (3.5.1 + 4.5.1)</t>
+  </si>
+  <si>
+    <t>05.2a. Amplitudenmodulation AM, SSB, CW (3.5.2 + 4.5.2)</t>
+  </si>
+  <si>
+    <t>05.3a. Frequenz- und Phasenmodulation (3.5.3 + 4.5.3)</t>
+  </si>
+  <si>
+    <t>05.4a. Digitale Übertragungsverfahren (3.5.4 + 4.5.4)</t>
+  </si>
+  <si>
+    <t>06.1a. Transceiver (3.6.1)</t>
+  </si>
+  <si>
+    <t>06.2a. Empfänger (3.6.2 + 4.6.1)</t>
+  </si>
+  <si>
+    <t>06.3a. Empfängerstufen (3.6.3 + 4.6.2)</t>
+  </si>
+  <si>
+    <t>06.4a. Sender und Senderstufen (3.6.4 + 4.6.3)</t>
+  </si>
+  <si>
+    <t>06.5a. Leistungsverstärker (4.6.4)</t>
+  </si>
+  <si>
+    <t>06.6a. Konverter und Transverter (4.6.5)</t>
+  </si>
+  <si>
+    <t>06.7a. Digitale Signalverarbeitung (4.6.6)</t>
+  </si>
+  <si>
+    <t>07.1a. Antennen (3.7.1 + 4.7.1)</t>
+  </si>
+  <si>
+    <t>07.2a. Antennenmerkmale (4.7.2)</t>
+  </si>
+  <si>
+    <t>07.3a. Übertragungsleitungen (3.7.2 + 4.7.3)</t>
+  </si>
+  <si>
+    <t>07.4a. Anpassung usw. (3.7.3)</t>
+  </si>
+  <si>
+    <t>07.5a. Strahlungsleistung  (3.7.4 + 4.7.5)</t>
+  </si>
+  <si>
+    <t>08.1a. Ionosphäre (3.8.1 + 4.8.1)</t>
+  </si>
+  <si>
+    <t>08.2a. Kurzwellenausbreitung (3.8.2 + 4.8.2)</t>
+  </si>
+  <si>
+    <t>08.3a. Wellenausbreitung oberhalb 30 MHz (3.8.3 + 4.8.3)</t>
+  </si>
+  <si>
+    <t>09.1a. Strom- und Spannungsmessgeräte (3.9.1 + 4.9.1)</t>
+  </si>
+  <si>
+    <t>10.1a. Störungen elektronischer Geräte (3.10.1 + 4.10.1)</t>
+  </si>
+  <si>
+    <t>10.2a. Unerwünschte Aussendungen (3.10.2 + 4.10.2)</t>
+  </si>
+  <si>
+    <t>10.3a. Störfestigkeit (3.11.1)</t>
+  </si>
+  <si>
+    <t>11.1a. Schutz von Personen (3.11.2 + 4.11.1)</t>
+  </si>
+  <si>
+    <t>11.2a. Sicherheit (3.11.3 + 4.11.2)</t>
+  </si>
+  <si>
+    <t>09.3a. Oszilloskop (3.9.4 + 4.9.3)</t>
+  </si>
+  <si>
+    <t>09.5a. Frequenzmessung (3.9.3 + 4.9.5)</t>
+  </si>
+  <si>
+    <t>09.2a. Vektorieller Netzwerk Analysator (4.9.2)</t>
+  </si>
+  <si>
+    <t>09.4a. Stehwellenmessgerät (3.9.2 + 4.9.4)</t>
+  </si>
+  <si>
+    <t>03.4a. Übertrager und Transformatoren (4.3.4)</t>
+  </si>
+  <si>
+    <t>03.5a. Diode (3.3.4 + 4.3.5)</t>
+  </si>
+  <si>
+    <t>07. Antennen und Übertragungsleitungen</t>
+  </si>
+  <si>
+    <t>02.7a. Ohmsches Gesetz und  Stromkreis (3.2.5 + 3.2.7)</t>
+  </si>
+  <si>
+    <t>02.8a. Leistung (3.2.6 + 4.2.5)</t>
+  </si>
+  <si>
+    <t>04.6a. Oszillator (3.4.2 + 4.4.5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prüfungsteil "Technische Kenntnisse" der Klasse N und E (Entry-License und Novice-License) </t>
+  </si>
+  <si>
+    <t>zu einem gemeinsamen Fragenkatalog zusammengeführt werden könnten.</t>
+  </si>
+  <si>
+    <t>Die Nummerierung der Kategorien ist so gewählt, dass DLE-2024 und DLA-2024</t>
+  </si>
+  <si>
+    <t>Nummerierung mit Lücken</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>= Frage auf Niveau NOVICE</t>
+  </si>
+  <si>
+    <t>b</t>
+  </si>
+  <si>
+    <t>= Fragen auf Niveau CEPT (aufbauend  auf 'a'-Fragen)</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>= Fragen aus den Niveaus NOVICE und CEPT gemischt</t>
+  </si>
+  <si>
+    <t>Die Buchstaben bei der Nummerierung geben einen Hinweis auf den Inhalt:</t>
+  </si>
+  <si>
+    <t>-- Dateiname darf nicht geändert werden.</t>
+  </si>
+  <si>
+    <t>-- Name des Reiters "Kategorie-Namen" darf nicht geändert werden.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -611,6 +629,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -632,7 +657,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -640,6 +665,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -944,7 +970,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.77734375" customWidth="1"/>
@@ -953,7 +979,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
-        <v>162</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -961,19 +987,19 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>174</v>
+        <v>118</v>
       </c>
       <c r="B3" s="4"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B4" s="4"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>173</v>
+        <v>117</v>
       </c>
       <c r="B5" s="4"/>
     </row>
@@ -982,7 +1008,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>168</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
@@ -990,48 +1016,92 @@
         <v>84</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>163</v>
+        <v>113</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>164</v>
+        <v>110</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>165</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>166</v>
+        <v>111</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>167</v>
-      </c>
+        <v>115</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B11" s="4"/>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>169</v>
-      </c>
+        <v>174</v>
+      </c>
+      <c r="B12" s="4"/>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>171</v>
-      </c>
+        <v>173</v>
+      </c>
+      <c r="B13" s="4"/>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>170</v>
-      </c>
+        <v>172</v>
+      </c>
+      <c r="B14" s="4"/>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B15" s="4"/>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" s="6" t="s">
+      <c r="A16" t="s">
+        <v>181</v>
+      </c>
+      <c r="B16" s="4"/>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>175</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
         <v>177</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>179</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" s="6" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" s="4" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="4" t="s">
+        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -1045,9 +1115,8 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.77734375" customWidth="1"/>
-    <col min="2" max="2" width="50.6640625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="50.6640625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="66.5546875" customWidth="1"/>
+    <col min="2" max="2" width="40.77734375" style="3" customWidth="1"/>
+    <col min="3" max="3" width="50.77734375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" s="5" customFormat="1" ht="18" x14ac:dyDescent="0.35">
@@ -1055,10 +1124,10 @@
         <v>84</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>160</v>
+        <v>110</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>161</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -1066,21 +1135,21 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>129</v>
+        <v>85</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>85</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>175</v>
+        <v>119</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>129</v>
+        <v>85</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>86</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -1088,10 +1157,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>129</v>
+        <v>85</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>86</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -1099,10 +1168,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>129</v>
+        <v>85</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>87</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -1110,10 +1179,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>130</v>
+        <v>86</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>88</v>
+        <v>124</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -1121,10 +1190,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>130</v>
+        <v>86</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>89</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -1132,10 +1201,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>130</v>
+        <v>86</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>90</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -1143,10 +1212,10 @@
         <v>4</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>130</v>
+        <v>86</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>90</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -1154,10 +1223,10 @@
         <v>5</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>130</v>
+        <v>86</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>90</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -1165,10 +1234,10 @@
         <v>8</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>130</v>
+        <v>86</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>90</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -1176,10 +1245,10 @@
         <v>9</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>130</v>
+        <v>86</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>91</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -1187,10 +1256,10 @@
         <v>10</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>130</v>
+        <v>86</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>91</v>
+        <v>127</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -1198,10 +1267,10 @@
         <v>11</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>130</v>
+        <v>86</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>92</v>
+        <v>168</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
@@ -1209,10 +1278,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>130</v>
+        <v>86</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>92</v>
+        <v>168</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
@@ -1220,10 +1289,10 @@
         <v>13</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>130</v>
+        <v>86</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>93</v>
+        <v>169</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -1231,10 +1300,10 @@
         <v>12</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>130</v>
+        <v>86</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>93</v>
+        <v>169</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
@@ -1242,10 +1311,10 @@
         <v>15</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>133</v>
+        <v>89</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>94</v>
+        <v>128</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
@@ -1253,10 +1322,10 @@
         <v>16</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>133</v>
+        <v>89</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>94</v>
+        <v>128</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -1264,10 +1333,10 @@
         <v>17</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>133</v>
+        <v>89</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>95</v>
+        <v>129</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
@@ -1275,10 +1344,10 @@
         <v>18</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>133</v>
+        <v>89</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>95</v>
+        <v>129</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
@@ -1286,10 +1355,10 @@
         <v>19</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>133</v>
+        <v>89</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>96</v>
+        <v>130</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
@@ -1297,43 +1366,43 @@
         <v>20</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>133</v>
+        <v>89</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>96</v>
+        <v>130</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>133</v>
+        <v>89</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>97</v>
+        <v>165</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>97</v>
+        <v>89</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>158</v>
+        <v>89</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
@@ -1341,10 +1410,10 @@
         <v>23</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>133</v>
+        <v>89</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>159</v>
+        <v>131</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
@@ -1352,10 +1421,10 @@
         <v>25</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>133</v>
+        <v>89</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>159</v>
+        <v>131</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
@@ -1363,10 +1432,10 @@
         <v>26</v>
       </c>
       <c r="B29" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>132</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
@@ -1374,10 +1443,10 @@
         <v>29</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>132</v>
+        <v>88</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>99</v>
+        <v>133</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
@@ -1385,10 +1454,10 @@
         <v>27</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>132</v>
+        <v>88</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>100</v>
+        <v>134</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
@@ -1396,10 +1465,10 @@
         <v>30</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>132</v>
+        <v>88</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>100</v>
+        <v>134</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
@@ -1407,10 +1476,10 @@
         <v>31</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>132</v>
+        <v>88</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>101</v>
+        <v>135</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
@@ -1418,10 +1487,10 @@
         <v>28</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>132</v>
+        <v>88</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>102</v>
+        <v>170</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
@@ -1429,10 +1498,10 @@
         <v>32</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>132</v>
+        <v>88</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>102</v>
+        <v>170</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
@@ -1440,10 +1509,10 @@
         <v>33</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>103</v>
+        <v>136</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
@@ -1451,10 +1520,10 @@
         <v>34</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>103</v>
+        <v>136</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
@@ -1462,10 +1531,10 @@
         <v>35</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>104</v>
+        <v>137</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
@@ -1473,10 +1542,10 @@
         <v>36</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>104</v>
+        <v>137</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
@@ -1484,10 +1553,10 @@
         <v>37</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>105</v>
+        <v>138</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
@@ -1495,10 +1564,10 @@
         <v>38</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>105</v>
+        <v>138</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
@@ -1506,10 +1575,10 @@
         <v>39</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>106</v>
+        <v>139</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
@@ -1517,10 +1586,10 @@
         <v>40</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>106</v>
+        <v>139</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
@@ -1528,10 +1597,10 @@
         <v>42</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>134</v>
+        <v>90</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>108</v>
+        <v>140</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
@@ -1539,10 +1608,10 @@
         <v>44</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>134</v>
+        <v>90</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>109</v>
+        <v>141</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
@@ -1550,10 +1619,10 @@
         <v>41</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>134</v>
+        <v>90</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>109</v>
+        <v>141</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
@@ -1561,10 +1630,10 @@
         <v>45</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>134</v>
+        <v>90</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>107</v>
+        <v>142</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
@@ -1572,10 +1641,10 @@
         <v>43</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>134</v>
+        <v>90</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>107</v>
+        <v>142</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
@@ -1583,10 +1652,10 @@
         <v>47</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>134</v>
+        <v>90</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>110</v>
+        <v>143</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
@@ -1594,10 +1663,10 @@
         <v>46</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>134</v>
+        <v>90</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>110</v>
+        <v>143</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
@@ -1605,10 +1674,10 @@
         <v>48</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>134</v>
+        <v>90</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>111</v>
+        <v>144</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
@@ -1616,10 +1685,10 @@
         <v>49</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>134</v>
+        <v>90</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>112</v>
+        <v>145</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
@@ -1627,10 +1696,10 @@
         <v>50</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>134</v>
+        <v>90</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>113</v>
+        <v>146</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
@@ -1638,10 +1707,10 @@
         <v>51</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>135</v>
+        <v>167</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>114</v>
+        <v>147</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
@@ -1649,10 +1718,10 @@
         <v>52</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>135</v>
+        <v>167</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>114</v>
+        <v>147</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
@@ -1660,10 +1729,10 @@
         <v>53</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>135</v>
+        <v>167</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>115</v>
+        <v>148</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
@@ -1671,10 +1740,10 @@
         <v>54</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>135</v>
+        <v>167</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>116</v>
+        <v>149</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
@@ -1682,10 +1751,10 @@
         <v>55</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>135</v>
+        <v>167</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>116</v>
+        <v>149</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
@@ -1693,10 +1762,10 @@
         <v>56</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>135</v>
+        <v>167</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>118</v>
+        <v>150</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
@@ -1704,10 +1773,10 @@
         <v>57</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>135</v>
+        <v>167</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>118</v>
+        <v>150</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
@@ -1715,10 +1784,10 @@
         <v>58</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>135</v>
+        <v>167</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>117</v>
+        <v>151</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
@@ -1726,10 +1795,10 @@
         <v>59</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>135</v>
+        <v>167</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>117</v>
+        <v>151</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
@@ -1737,10 +1806,10 @@
         <v>60</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>136</v>
+        <v>91</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>119</v>
+        <v>152</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
@@ -1748,10 +1817,10 @@
         <v>61</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>136</v>
+        <v>91</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>119</v>
+        <v>152</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
@@ -1759,10 +1828,10 @@
         <v>62</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>136</v>
+        <v>91</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>120</v>
+        <v>153</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.3">
@@ -1770,10 +1839,10 @@
         <v>63</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>136</v>
+        <v>91</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>120</v>
+        <v>153</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.3">
@@ -1781,10 +1850,10 @@
         <v>64</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>136</v>
+        <v>91</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>121</v>
+        <v>154</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
@@ -1792,10 +1861,10 @@
         <v>65</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>136</v>
+        <v>91</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>121</v>
+        <v>154</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
@@ -1803,10 +1872,10 @@
         <v>66</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>137</v>
+        <v>92</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>122</v>
+        <v>155</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.3">
@@ -1814,87 +1883,87 @@
         <v>67</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>143</v>
+        <v>95</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>122</v>
+        <v>155</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>144</v>
+        <v>98</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>123</v>
+        <v>163</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A72" t="s">
-        <v>73</v>
+      <c r="A72" s="7" t="s">
+        <v>72</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="C72" s="3" t="s">
-        <v>123</v>
+        <v>101</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="C73" s="2" t="s">
-        <v>124</v>
+        <v>102</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A74" t="s">
-        <v>70</v>
+      <c r="A74" s="7" t="s">
+        <v>68</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>147</v>
+        <v>96</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>125</v>
+        <v>164</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>148</v>
+        <v>97</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>125</v>
+        <v>164</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A76" t="s">
-        <v>72</v>
+      <c r="A76" s="7" t="s">
+        <v>70</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>149</v>
+        <v>99</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>126</v>
+        <v>162</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>126</v>
+        <v>162</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.3">
@@ -1902,10 +1971,10 @@
         <v>75</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>138</v>
+        <v>93</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>127</v>
+        <v>156</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.3">
@@ -1913,10 +1982,10 @@
         <v>76</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>151</v>
+        <v>103</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>127</v>
+        <v>156</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.3">
@@ -1924,10 +1993,10 @@
         <v>77</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>152</v>
+        <v>104</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>128</v>
+        <v>157</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.3">
@@ -1935,10 +2004,10 @@
         <v>78</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>153</v>
+        <v>105</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>128</v>
+        <v>157</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.3">
@@ -1946,10 +2015,10 @@
         <v>79</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>154</v>
+        <v>106</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>140</v>
+        <v>158</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.3">
@@ -1957,10 +2026,10 @@
         <v>81</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>139</v>
+        <v>94</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>141</v>
+        <v>159</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.3">
@@ -1968,10 +2037,10 @@
         <v>80</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>155</v>
+        <v>107</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>141</v>
+        <v>159</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.3">
@@ -1979,10 +2048,10 @@
         <v>83</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>156</v>
+        <v>108</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>142</v>
+        <v>160</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.3">
@@ -1990,10 +2059,10 @@
         <v>82</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>157</v>
+        <v>109</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>142</v>
+        <v>160</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>